<commit_message>
Updated description, outcome message and added  to output variables.
</commit_message>
<xml_diff>
--- a/rules/CORE-000552/negative/01/data/unit-test-coreid-CG0220-negative 1.xlsx
+++ b/rules/CORE-000552/negative/01/data/unit-test-coreid-CG0220-negative 1.xlsx
@@ -37,7 +37,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" mc:Ignorable="x14ac">
   <numFmts count="0"/>
-  <fonts count="11" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
@@ -54,7 +54,6 @@
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
-      <i/>
     </font>
     <font>
       <sz val="11"/>
@@ -65,28 +64,8 @@
       <sz val="11"/>
       <name val="Calibri"/>
     </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
   </fonts>
-  <fills count="9">
+  <fills count="4">
     <fill>
       <patternFill patternType="none">
         <bgColor/>
@@ -100,34 +79,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00FFFFCC"/>
-        <bgColor/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFFFCC"/>
-        <bgColor/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <bgColor/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <bgColor/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF00"/>
-        <bgColor/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF00"/>
         <bgColor/>
       </patternFill>
     </fill>
@@ -157,19 +108,14 @@
   <cellStyleXfs>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="1" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="8" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="9" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="10" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -512,10 +458,10 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="str">
+      <c r="A2" s="4" t="str">
         <v>sdtmig</v>
       </c>
-      <c r="B2" s="2" t="str">
+      <c r="B2" s="4" t="str">
         <v>3-4</v>
       </c>
     </row>
@@ -539,18 +485,18 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="str">
+      <c r="A2" s="4" t="str">
         <v>dm.xpt</v>
       </c>
-      <c r="B2" s="2" t="str">
+      <c r="B2" s="4" t="str">
         <v>Demographics</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="str">
+      <c r="A3" s="4" t="str">
         <v>cm.xpt</v>
       </c>
-      <c r="B3" s="2" t="str">
+      <c r="B3" s="4" t="str">
         <v>Concomitant/Prior Medications</v>
       </c>
     </row>
@@ -563,7 +509,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F10"/>
+  <dimension ref="A1:F13"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="3" t="str">
@@ -586,39 +532,39 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2">
+      <c r="A2" s="4">
         <v>1</v>
       </c>
-      <c r="B2" s="2" t="str">
+      <c r="B2" s="4" t="str">
         <v>cm.xpt</v>
       </c>
-      <c r="C2" s="2" t="str">
+      <c r="C2" s="4" t="str">
         <v>Record</v>
       </c>
-      <c r="D2" s="2">
+      <c r="D2" s="4">
         <v>11</v>
       </c>
-      <c r="E2" s="2" t="str">
+      <c r="E2" s="4" t="str">
         <v>CMSTDTC</v>
       </c>
-      <c r="F2" s="2" t="str">
+      <c r="F2" s="4" t="str">
         <v>2013-02-18</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2">
+      <c r="A3" s="4">
         <v>1</v>
       </c>
-      <c r="B3" s="2" t="str">
+      <c r="B3" s="4" t="str">
         <v>cm.xpt</v>
       </c>
-      <c r="C3" s="2" t="str">
+      <c r="C3" s="4" t="str">
         <v>Record</v>
       </c>
-      <c r="D3" s="2">
+      <c r="D3" s="4">
         <v>11</v>
       </c>
-      <c r="E3" s="2" t="str">
+      <c r="E3" s="4" t="str">
         <v>CMSTDY</v>
       </c>
     </row>
@@ -627,7 +573,7 @@
         <v>1</v>
       </c>
       <c r="B4" s="2" t="str">
-        <v>dm.xpt</v>
+        <v>cm.xpt</v>
       </c>
       <c r="C4" s="2" t="str">
         <v>Record</v>
@@ -636,75 +582,75 @@
         <v>11</v>
       </c>
       <c r="E4" s="2" t="str">
+        <v>$val_stdy</v>
+      </c>
+      <c r="F4" s="2">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4">
+        <v>1</v>
+      </c>
+      <c r="B5" s="4" t="str">
+        <v>dm.xpt</v>
+      </c>
+      <c r="C5" s="4" t="str">
+        <v>Record</v>
+      </c>
+      <c r="D5" s="4">
+        <v>11</v>
+      </c>
+      <c r="E5" s="4" t="str">
         <v>RFSTDTC</v>
       </c>
-      <c r="F4" s="2" t="str">
+      <c r="F5" s="4" t="str">
         <v>2013-01-05</v>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="2">
+    <row r="6">
+      <c r="A6" s="4">
         <v>2</v>
       </c>
-      <c r="B5" s="2" t="str">
+      <c r="B6" s="4" t="str">
         <v>cm.xpt</v>
       </c>
-      <c r="C5" s="2" t="str">
+      <c r="C6" s="4" t="str">
         <v>Record</v>
       </c>
-      <c r="D5" s="2">
+      <c r="D6" s="4">
         <v>12</v>
       </c>
-      <c r="E5" s="2" t="str">
+      <c r="E6" s="4" t="str">
         <v>CMSTDTC</v>
       </c>
-      <c r="F5" s="2" t="str">
+      <c r="F6" s="4" t="str">
         <v>2013-02-18</v>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="2">
+    <row r="7">
+      <c r="A7" s="4">
         <v>2</v>
       </c>
-      <c r="B6" s="2" t="str">
+      <c r="B7" s="4" t="str">
         <v>cm.xpt</v>
       </c>
-      <c r="C6" s="2" t="str">
+      <c r="C7" s="4" t="str">
         <v>Record</v>
       </c>
-      <c r="D6" s="2">
+      <c r="D7" s="4">
         <v>12</v>
       </c>
-      <c r="E6" s="2" t="str">
+      <c r="E7" s="4" t="str">
         <v>CMSTDY</v>
       </c>
-      <c r="F6" s="2">
+      <c r="F7" s="4">
         <v>45</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="2">
-        <v>2</v>
-      </c>
-      <c r="B7" s="2" t="str">
-        <v>dm.xpt</v>
-      </c>
-      <c r="C7" s="2" t="str">
-        <v>Record</v>
-      </c>
-      <c r="D7" s="2">
-        <v>12</v>
-      </c>
-      <c r="E7" s="2" t="str">
-        <v>RFSTDTC</v>
-      </c>
-      <c r="F7" s="2" t="str">
-        <v>2014-05-11</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B8" s="2" t="str">
         <v>cm.xpt</v>
@@ -713,58 +659,118 @@
         <v>Record</v>
       </c>
       <c r="D8" s="2">
+        <v>12</v>
+      </c>
+      <c r="E8" s="2" t="str">
+        <v>$val_stdy</v>
+      </c>
+      <c r="F8" s="2">
+        <v>-447</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4">
+        <v>2</v>
+      </c>
+      <c r="B9" s="4" t="str">
+        <v>dm.xpt</v>
+      </c>
+      <c r="C9" s="4" t="str">
+        <v>Record</v>
+      </c>
+      <c r="D9" s="4">
+        <v>12</v>
+      </c>
+      <c r="E9" s="4" t="str">
+        <v>RFSTDTC</v>
+      </c>
+      <c r="F9" s="4" t="str">
+        <v>2014-05-11</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4">
+        <v>3</v>
+      </c>
+      <c r="B10" s="4" t="str">
+        <v>cm.xpt</v>
+      </c>
+      <c r="C10" s="4" t="str">
+        <v>Record</v>
+      </c>
+      <c r="D10" s="4">
         <v>14</v>
       </c>
-      <c r="E8" s="2" t="str">
+      <c r="E10" s="4" t="str">
         <v>CMSTDTC</v>
       </c>
-      <c r="F8" s="2" t="str">
+      <c r="F10" s="4" t="str">
         <v>2011-07-15</v>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="2">
+    <row r="11">
+      <c r="A11" s="4">
         <v>3</v>
       </c>
-      <c r="B9" s="2" t="str">
+      <c r="B11" s="4" t="str">
         <v>cm.xpt</v>
       </c>
-      <c r="C9" s="2" t="str">
+      <c r="C11" s="4" t="str">
         <v>Record</v>
       </c>
-      <c r="D9" s="2">
+      <c r="D11" s="4">
         <v>14</v>
       </c>
-      <c r="E9" s="2" t="str">
+      <c r="E11" s="4" t="str">
         <v>CMSTDY</v>
       </c>
-      <c r="F9" s="2">
+      <c r="F11" s="4">
         <v>-511</v>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="2">
+    <row r="12">
+      <c r="A12" s="2">
         <v>3</v>
       </c>
-      <c r="B10" s="2" t="str">
+      <c r="B12" s="2" t="str">
+        <v>cm.xpt</v>
+      </c>
+      <c r="C12" s="2" t="str">
+        <v>Record</v>
+      </c>
+      <c r="D12" s="2">
+        <v>14</v>
+      </c>
+      <c r="E12" s="2" t="str">
+        <v>$val_stdy</v>
+      </c>
+      <c r="F12" s="2">
+        <v>-799</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4">
+        <v>3</v>
+      </c>
+      <c r="B13" s="4" t="str">
         <v>dm.xpt</v>
       </c>
-      <c r="C10" s="2" t="str">
+      <c r="C13" s="4" t="str">
         <v>Record</v>
       </c>
-      <c r="D10" s="2">
+      <c r="D13" s="4">
         <v>14</v>
       </c>
-      <c r="E10" s="2" t="str">
+      <c r="E13" s="4" t="str">
         <v>RFSTDTC</v>
       </c>
-      <c r="F10" s="2" t="str">
+      <c r="F13" s="4" t="str">
         <v>2013-09-21</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F10"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F13"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -854,7 +860,7 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="4" t="str">
+      <c r="A2" s="5" t="str">
         <v>Study Identifier</v>
       </c>
       <c r="B2" s="5" t="str">
@@ -1094,802 +1100,802 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="6" t="str">
+      <c r="A5" s="4" t="str">
         <v>CDISCPILOT01</v>
       </c>
-      <c r="B5" s="6" t="str">
+      <c r="B5" s="4" t="str">
         <v>DM</v>
       </c>
-      <c r="C5" s="6" t="str">
+      <c r="C5" s="4" t="str">
         <v>CDISC001</v>
       </c>
-      <c r="D5" s="6">
+      <c r="D5" s="4">
         <v>1115</v>
       </c>
-      <c r="E5" s="6" t="str">
-        <v/>
-      </c>
-      <c r="F5" s="6" t="str">
+      <c r="E5" s="4" t="str">
+        <v/>
+      </c>
+      <c r="F5" s="4" t="str">
         <v>2013-01-23</v>
       </c>
-      <c r="G5" s="6" t="str">
+      <c r="G5" s="4" t="str">
         <v>2012-11-30</v>
       </c>
-      <c r="H5" s="6" t="str">
+      <c r="H5" s="4" t="str">
         <v>2013-01-23</v>
       </c>
-      <c r="I5" s="6" t="str">
+      <c r="I5" s="4" t="str">
         <v>2012-11-23</v>
       </c>
-      <c r="J5" s="6" t="str">
+      <c r="J5" s="4" t="str">
         <v>2013-05-20</v>
       </c>
-      <c r="K5" s="2" t="str">
-        <v/>
-      </c>
-      <c r="L5" s="6" t="str">
-        <v/>
-      </c>
-      <c r="M5" s="6">
+      <c r="K5" s="4" t="str">
+        <v/>
+      </c>
+      <c r="L5" s="4" t="str">
+        <v/>
+      </c>
+      <c r="M5" s="4">
         <v>701</v>
       </c>
-      <c r="N5" s="6">
+      <c r="N5" s="4">
         <v>1928</v>
       </c>
-      <c r="O5" s="6">
+      <c r="O5" s="4">
         <v>84</v>
       </c>
-      <c r="P5" s="6" t="str">
+      <c r="P5" s="4" t="str">
         <v>YEARS</v>
       </c>
-      <c r="Q5" s="6" t="str">
+      <c r="Q5" s="4" t="str">
         <v>M</v>
       </c>
-      <c r="R5" s="6" t="str">
+      <c r="R5" s="4" t="str">
         <v>WHITE</v>
       </c>
-      <c r="S5" s="6" t="str">
+      <c r="S5" s="4" t="str">
         <v>NOT HISPANIC OR LATINO</v>
       </c>
-      <c r="T5" s="6" t="str">
+      <c r="T5" s="4" t="str">
         <v>ZAN_LOW</v>
       </c>
-      <c r="U5" s="6" t="str">
+      <c r="U5" s="4" t="str">
         <v>Zanomaline Low Dose (54 mg)</v>
       </c>
-      <c r="V5" s="6" t="str">
+      <c r="V5" s="4" t="str">
         <v>ZAN_LOW</v>
       </c>
-      <c r="W5" s="6" t="str">
+      <c r="W5" s="4" t="str">
         <v>Zanomaline Low Dose (54 mg)</v>
       </c>
-      <c r="X5" s="6" t="str">
-        <v/>
-      </c>
-      <c r="Y5" s="6" t="str">
-        <v/>
-      </c>
-      <c r="Z5" s="6" t="str">
+      <c r="X5" s="4" t="str">
+        <v/>
+      </c>
+      <c r="Y5" s="4" t="str">
+        <v/>
+      </c>
+      <c r="Z5" s="4" t="str">
         <v>USA</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="7" t="str">
+      <c r="A6" s="4" t="str">
         <v>CDISCPILOT01</v>
       </c>
-      <c r="B6" s="8" t="str">
+      <c r="B6" s="4" t="str">
         <v>DM</v>
       </c>
-      <c r="C6" s="8" t="str">
+      <c r="C6" s="4" t="str">
         <v>CDISC002</v>
       </c>
-      <c r="D6" s="8">
+      <c r="D6" s="4">
         <v>1211</v>
       </c>
-      <c r="E6" s="8" t="str">
-        <v/>
-      </c>
-      <c r="F6" s="8" t="str">
+      <c r="E6" s="4" t="str">
+        <v/>
+      </c>
+      <c r="F6" s="4" t="str">
         <v>2013-01-14</v>
       </c>
-      <c r="G6" s="8" t="str">
+      <c r="G6" s="4" t="str">
         <v>2012-11-15</v>
       </c>
-      <c r="H6" s="8" t="str">
+      <c r="H6" s="4" t="str">
         <v>2013-01-12</v>
       </c>
-      <c r="I6" s="8" t="str">
+      <c r="I6" s="4" t="str">
         <v>2012-10-30</v>
       </c>
-      <c r="J6" s="8" t="str">
+      <c r="J6" s="4" t="str">
         <v>2013-01-14</v>
       </c>
-      <c r="K6" s="8" t="str">
+      <c r="K6" s="4" t="str">
         <v>2013-01-14</v>
       </c>
-      <c r="L6" s="8" t="str">
+      <c r="L6" s="4" t="str">
         <v>Y</v>
       </c>
-      <c r="M6" s="8">
+      <c r="M6" s="4">
         <v>701</v>
       </c>
-      <c r="N6" s="8">
+      <c r="N6" s="4">
         <v>1936</v>
       </c>
-      <c r="O6" s="8">
+      <c r="O6" s="4">
         <v>76</v>
       </c>
-      <c r="P6" s="8" t="str">
+      <c r="P6" s="4" t="str">
         <v>YEARS</v>
       </c>
-      <c r="Q6" s="8" t="str">
+      <c r="Q6" s="4" t="str">
         <v>F</v>
       </c>
-      <c r="R6" s="8" t="str">
+      <c r="R6" s="4" t="str">
         <v>WHITE</v>
       </c>
-      <c r="S6" s="8" t="str">
+      <c r="S6" s="4" t="str">
         <v>NOT HISPANIC OR LATINO</v>
       </c>
-      <c r="T6" s="8" t="str">
+      <c r="T6" s="4" t="str">
         <v>ZAN_LOW</v>
       </c>
-      <c r="U6" s="8" t="str">
+      <c r="U6" s="4" t="str">
         <v>Zanomaline Low Dose (54 mg)</v>
       </c>
-      <c r="V6" s="8" t="str">
+      <c r="V6" s="4" t="str">
         <v>ZAN_LOW</v>
       </c>
-      <c r="W6" s="8" t="str">
+      <c r="W6" s="4" t="str">
         <v>Zanomaline Low Dose (54 mg)</v>
       </c>
-      <c r="X6" s="8" t="str">
-        <v/>
-      </c>
-      <c r="Y6" s="8" t="str">
-        <v/>
-      </c>
-      <c r="Z6" s="8" t="str">
+      <c r="X6" s="4" t="str">
+        <v/>
+      </c>
+      <c r="Y6" s="4" t="str">
+        <v/>
+      </c>
+      <c r="Z6" s="4" t="str">
         <v>USA</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="6" t="str">
+      <c r="A7" s="4" t="str">
         <v>CDISCPILOT01</v>
       </c>
-      <c r="B7" s="6" t="str">
+      <c r="B7" s="4" t="str">
         <v>DM</v>
       </c>
-      <c r="C7" s="6" t="str">
+      <c r="C7" s="4" t="str">
         <v>CDISC003</v>
       </c>
-      <c r="D7" s="6">
+      <c r="D7" s="4">
         <v>1302</v>
       </c>
-      <c r="E7" s="6" t="str">
-        <v/>
-      </c>
-      <c r="F7" s="6" t="str">
+      <c r="E7" s="4" t="str">
+        <v/>
+      </c>
+      <c r="F7" s="4" t="str">
         <v>2013-11-05</v>
       </c>
-      <c r="G7" s="6" t="str">
+      <c r="G7" s="4" t="str">
         <v>2013-08-29</v>
       </c>
-      <c r="H7" s="6" t="str">
+      <c r="H7" s="4" t="str">
         <v>2013-11-05</v>
       </c>
-      <c r="I7" s="6" t="str">
+      <c r="I7" s="4" t="str">
         <v>2013-08-20</v>
       </c>
-      <c r="J7" s="6" t="str">
+      <c r="J7" s="4" t="str">
         <v>2014-02-13</v>
       </c>
-      <c r="K7" s="2" t="str">
-        <v/>
-      </c>
-      <c r="L7" s="6" t="str">
-        <v/>
-      </c>
-      <c r="M7" s="6">
+      <c r="K7" s="4" t="str">
+        <v/>
+      </c>
+      <c r="L7" s="4" t="str">
+        <v/>
+      </c>
+      <c r="M7" s="4">
         <v>701</v>
       </c>
-      <c r="N7" s="6">
+      <c r="N7" s="4">
         <v>1951</v>
       </c>
-      <c r="O7" s="6">
+      <c r="O7" s="4">
         <v>61</v>
       </c>
-      <c r="P7" s="6" t="str">
+      <c r="P7" s="4" t="str">
         <v>YEARS</v>
       </c>
-      <c r="Q7" s="6" t="str">
+      <c r="Q7" s="4" t="str">
         <v>M</v>
       </c>
-      <c r="R7" s="6" t="str">
+      <c r="R7" s="4" t="str">
         <v>WHITE</v>
       </c>
-      <c r="S7" s="6" t="str">
+      <c r="S7" s="4" t="str">
         <v>NOT HISPANIC OR LATINO</v>
       </c>
-      <c r="T7" s="6" t="str">
+      <c r="T7" s="4" t="str">
         <v>ZAN_HIGH</v>
       </c>
-      <c r="U7" s="6" t="str">
+      <c r="U7" s="4" t="str">
         <v>Zanomaline High Dose (81 mg)</v>
       </c>
-      <c r="V7" s="6" t="str">
+      <c r="V7" s="4" t="str">
         <v>ZAN_HIGH</v>
       </c>
-      <c r="W7" s="6" t="str">
+      <c r="W7" s="4" t="str">
         <v>Zanomaline High Dose (81 mg)</v>
       </c>
-      <c r="X7" s="6" t="str">
-        <v/>
-      </c>
-      <c r="Y7" s="6" t="str">
-        <v/>
-      </c>
-      <c r="Z7" s="6" t="str">
+      <c r="X7" s="4" t="str">
+        <v/>
+      </c>
+      <c r="Y7" s="4" t="str">
+        <v/>
+      </c>
+      <c r="Z7" s="4" t="str">
         <v>USA</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="8" t="str">
+      <c r="A8" s="4" t="str">
         <v>CDISCPILOT01</v>
       </c>
-      <c r="B8" s="8" t="str">
+      <c r="B8" s="4" t="str">
         <v>DM</v>
       </c>
-      <c r="C8" s="8" t="str">
+      <c r="C8" s="4" t="str">
         <v>CDISC004</v>
       </c>
-      <c r="D8" s="8">
+      <c r="D8" s="4">
         <v>1345</v>
       </c>
-      <c r="E8" s="8" t="str">
-        <v/>
-      </c>
-      <c r="F8" s="8" t="str">
+      <c r="E8" s="4" t="str">
+        <v/>
+      </c>
+      <c r="F8" s="4" t="str">
         <v>2014-03-18</v>
       </c>
-      <c r="G8" s="8" t="str">
+      <c r="G8" s="4" t="str">
         <v>2013-10-08</v>
       </c>
-      <c r="H8" s="8" t="str">
+      <c r="H8" s="4" t="str">
         <v>2014-03-18</v>
       </c>
-      <c r="I8" s="8" t="str">
+      <c r="I8" s="4" t="str">
         <v>2013-10-01</v>
       </c>
-      <c r="J8" s="8" t="str">
+      <c r="J8" s="4" t="str">
         <v>2014-03-18</v>
       </c>
-      <c r="K8" s="8" t="str">
-        <v/>
-      </c>
-      <c r="L8" s="8" t="str">
-        <v/>
-      </c>
-      <c r="M8" s="8">
+      <c r="K8" s="4" t="str">
+        <v/>
+      </c>
+      <c r="L8" s="4" t="str">
+        <v/>
+      </c>
+      <c r="M8" s="4">
         <v>701</v>
       </c>
-      <c r="N8" s="8">
+      <c r="N8" s="4">
         <v>1950</v>
       </c>
-      <c r="O8" s="8">
+      <c r="O8" s="4">
         <v>63</v>
       </c>
-      <c r="P8" s="8" t="str">
+      <c r="P8" s="4" t="str">
         <v>YEARS</v>
       </c>
-      <c r="Q8" s="8" t="str">
+      <c r="Q8" s="4" t="str">
         <v>F</v>
       </c>
-      <c r="R8" s="8" t="str">
+      <c r="R8" s="4" t="str">
         <v>WHITE</v>
       </c>
-      <c r="S8" s="8" t="str">
+      <c r="S8" s="4" t="str">
         <v>NOT HISPANIC OR LATINO</v>
       </c>
-      <c r="T8" s="8" t="str">
-        <v/>
-      </c>
-      <c r="U8" s="8" t="str">
-        <v/>
-      </c>
-      <c r="V8" s="8" t="str">
-        <v/>
-      </c>
-      <c r="W8" s="8" t="str">
-        <v/>
-      </c>
-      <c r="X8" s="8" t="str">
+      <c r="T8" s="4" t="str">
+        <v/>
+      </c>
+      <c r="U8" s="4" t="str">
+        <v/>
+      </c>
+      <c r="V8" s="4" t="str">
+        <v/>
+      </c>
+      <c r="W8" s="4" t="str">
+        <v/>
+      </c>
+      <c r="X8" s="4" t="str">
         <v>SCREEN FAILURE</v>
       </c>
-      <c r="Y8" s="8" t="str">
-        <v/>
-      </c>
-      <c r="Z8" s="8" t="str">
+      <c r="Y8" s="4" t="str">
+        <v/>
+      </c>
+      <c r="Z8" s="4" t="str">
         <v>USA</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="6" t="str">
+      <c r="A9" s="4" t="str">
         <v>CDISCPILOT01</v>
       </c>
-      <c r="B9" s="6" t="str">
+      <c r="B9" s="4" t="str">
         <v>DM</v>
       </c>
-      <c r="C9" s="6" t="str">
+      <c r="C9" s="4" t="str">
         <v>CDISC005</v>
       </c>
-      <c r="D9" s="6">
+      <c r="D9" s="4">
         <v>1383</v>
       </c>
-      <c r="E9" s="6" t="str">
-        <v/>
-      </c>
-      <c r="F9" s="6" t="str">
+      <c r="E9" s="4" t="str">
+        <v/>
+      </c>
+      <c r="F9" s="4" t="str">
         <v>2013-08-06</v>
       </c>
-      <c r="G9" s="6" t="str">
+      <c r="G9" s="4" t="str">
         <v>2013-02-04</v>
       </c>
-      <c r="H9" s="6" t="str">
+      <c r="H9" s="4" t="str">
         <v>2013-08-06</v>
       </c>
-      <c r="I9" s="6" t="str">
+      <c r="I9" s="4" t="str">
         <v>2013-01-22</v>
       </c>
-      <c r="J9" s="6" t="str">
+      <c r="J9" s="4" t="str">
         <v>2013-08-06</v>
       </c>
-      <c r="K9" s="2" t="str">
-        <v/>
-      </c>
-      <c r="L9" s="6" t="str">
-        <v/>
-      </c>
-      <c r="M9" s="6">
+      <c r="K9" s="4" t="str">
+        <v/>
+      </c>
+      <c r="L9" s="4" t="str">
+        <v/>
+      </c>
+      <c r="M9" s="4">
         <v>701</v>
       </c>
-      <c r="N9" s="6">
+      <c r="N9" s="4">
         <v>1941</v>
       </c>
-      <c r="O9" s="6">
+      <c r="O9" s="4">
         <v>72</v>
       </c>
-      <c r="P9" s="6" t="str">
+      <c r="P9" s="4" t="str">
         <v>YEARS</v>
       </c>
-      <c r="Q9" s="6" t="str">
+      <c r="Q9" s="4" t="str">
         <v>F</v>
       </c>
-      <c r="R9" s="6" t="str">
+      <c r="R9" s="4" t="str">
         <v>WHITE</v>
       </c>
-      <c r="S9" s="6" t="str">
+      <c r="S9" s="4" t="str">
         <v>NOT HISPANIC OR LATINO</v>
       </c>
-      <c r="T9" s="6" t="str">
+      <c r="T9" s="4" t="str">
         <v>ZAN_HIGH</v>
       </c>
-      <c r="U9" s="6" t="str">
+      <c r="U9" s="4" t="str">
         <v>Zanomaline High Dose (81 mg)</v>
       </c>
-      <c r="V9" s="6" t="str">
-        <v/>
-      </c>
-      <c r="W9" s="6" t="str">
-        <v/>
-      </c>
-      <c r="X9" s="6" t="str">
+      <c r="V9" s="4" t="str">
+        <v/>
+      </c>
+      <c r="W9" s="4" t="str">
+        <v/>
+      </c>
+      <c r="X9" s="4" t="str">
         <v>NOT TREATED</v>
       </c>
-      <c r="Y9" s="6" t="str">
-        <v/>
-      </c>
-      <c r="Z9" s="6" t="str">
+      <c r="Y9" s="4" t="str">
+        <v/>
+      </c>
+      <c r="Z9" s="4" t="str">
         <v>USA</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="8" t="str">
+      <c r="A10" s="4" t="str">
         <v>CDISCPILOT01</v>
       </c>
-      <c r="B10" s="8" t="str">
+      <c r="B10" s="4" t="str">
         <v>DM</v>
       </c>
-      <c r="C10" s="8" t="str">
+      <c r="C10" s="4" t="str">
         <v>CDISC006</v>
       </c>
-      <c r="D10" s="8">
+      <c r="D10" s="4">
         <v>1429</v>
       </c>
-      <c r="E10" s="8" t="str">
-        <v/>
-      </c>
-      <c r="F10" s="8" t="str">
+      <c r="E10" s="4" t="str">
+        <v/>
+      </c>
+      <c r="F10" s="4" t="str">
         <v>2013-04-30</v>
       </c>
-      <c r="G10" s="8" t="str">
+      <c r="G10" s="4" t="str">
         <v>2013-03-19</v>
       </c>
-      <c r="H10" s="8" t="str">
+      <c r="H10" s="4" t="str">
         <v>2013-04-30</v>
       </c>
-      <c r="I10" s="8" t="str">
+      <c r="I10" s="4" t="str">
         <v>2013-02-25</v>
       </c>
-      <c r="J10" s="8" t="str">
+      <c r="J10" s="4" t="str">
         <v>2013-04-30</v>
       </c>
-      <c r="K10" s="8" t="str">
-        <v/>
-      </c>
-      <c r="L10" s="8" t="str">
-        <v/>
-      </c>
-      <c r="M10" s="8">
+      <c r="K10" s="4" t="str">
+        <v/>
+      </c>
+      <c r="L10" s="4" t="str">
+        <v/>
+      </c>
+      <c r="M10" s="4">
         <v>701</v>
       </c>
-      <c r="N10" s="8">
+      <c r="N10" s="4">
         <v>1929</v>
       </c>
-      <c r="O10" s="8">
+      <c r="O10" s="4">
         <v>84</v>
       </c>
-      <c r="P10" s="8" t="str">
+      <c r="P10" s="4" t="str">
         <v>YEARS</v>
       </c>
-      <c r="Q10" s="8" t="str">
+      <c r="Q10" s="4" t="str">
         <v>F</v>
       </c>
-      <c r="R10" s="8" t="str">
+      <c r="R10" s="4" t="str">
         <v>WHITE</v>
       </c>
-      <c r="S10" s="8" t="str">
+      <c r="S10" s="4" t="str">
         <v>NOT HISPANIC OR LATINO</v>
       </c>
-      <c r="T10" s="8" t="str">
-        <v/>
-      </c>
-      <c r="U10" s="8" t="str">
-        <v/>
-      </c>
-      <c r="V10" s="8" t="str">
-        <v/>
-      </c>
-      <c r="W10" s="8" t="str">
-        <v/>
-      </c>
-      <c r="X10" s="8" t="str">
+      <c r="T10" s="4" t="str">
+        <v/>
+      </c>
+      <c r="U10" s="4" t="str">
+        <v/>
+      </c>
+      <c r="V10" s="4" t="str">
+        <v/>
+      </c>
+      <c r="W10" s="4" t="str">
+        <v/>
+      </c>
+      <c r="X10" s="4" t="str">
         <v>NOT ASSIGNED</v>
       </c>
-      <c r="Y10" s="8" t="str">
-        <v/>
-      </c>
-      <c r="Z10" s="8" t="str">
+      <c r="Y10" s="4" t="str">
+        <v/>
+      </c>
+      <c r="Z10" s="4" t="str">
         <v>USA</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="6" t="str">
+      <c r="A11" s="4" t="str">
         <v>CDISCPILOT01</v>
       </c>
-      <c r="B11" s="6" t="str">
+      <c r="B11" s="4" t="str">
         <v>DM</v>
       </c>
-      <c r="C11" s="6" t="str">
+      <c r="C11" s="4" t="str">
         <v>CDISC007</v>
       </c>
-      <c r="D11" s="6">
+      <c r="D11" s="4">
         <v>1444</v>
       </c>
-      <c r="E11" s="9" t="str">
+      <c r="E11" s="6" t="str">
         <v>2013-01-05</v>
       </c>
-      <c r="F11" s="6" t="str">
+      <c r="F11" s="4" t="str">
         <v>2013-02-13</v>
       </c>
-      <c r="G11" s="6" t="str">
+      <c r="G11" s="4" t="str">
         <v>2013-01-05</v>
       </c>
-      <c r="H11" s="6" t="str">
+      <c r="H11" s="4" t="str">
         <v>2013-02-12</v>
       </c>
-      <c r="I11" s="6" t="str">
+      <c r="I11" s="4" t="str">
         <v>2012-12-31</v>
       </c>
-      <c r="J11" s="6" t="str">
+      <c r="J11" s="4" t="str">
         <v>2013-06-20</v>
       </c>
-      <c r="K11" s="2" t="str">
-        <v/>
-      </c>
-      <c r="L11" s="6" t="str">
-        <v/>
-      </c>
-      <c r="M11" s="6">
+      <c r="K11" s="4" t="str">
+        <v/>
+      </c>
+      <c r="L11" s="4" t="str">
+        <v/>
+      </c>
+      <c r="M11" s="4">
         <v>701</v>
       </c>
-      <c r="N11" s="6">
+      <c r="N11" s="4">
         <v>1949</v>
       </c>
-      <c r="O11" s="6">
+      <c r="O11" s="4">
         <v>63</v>
       </c>
-      <c r="P11" s="6" t="str">
+      <c r="P11" s="4" t="str">
         <v>YEARS</v>
       </c>
-      <c r="Q11" s="6" t="str">
+      <c r="Q11" s="4" t="str">
         <v>M</v>
       </c>
-      <c r="R11" s="6" t="str">
+      <c r="R11" s="4" t="str">
         <v>WHITE</v>
       </c>
-      <c r="S11" s="6" t="str">
+      <c r="S11" s="4" t="str">
         <v>HISPANIC OR LATINO</v>
       </c>
-      <c r="T11" s="6" t="str">
+      <c r="T11" s="4" t="str">
         <v>ZAN_HIGH</v>
       </c>
-      <c r="U11" s="6" t="str">
+      <c r="U11" s="4" t="str">
         <v>Zanomaline High Dose (81 mg)</v>
       </c>
-      <c r="V11" s="6" t="str">
+      <c r="V11" s="4" t="str">
         <v>ZAN_HIGH</v>
       </c>
-      <c r="W11" s="6" t="str">
-        <v/>
-      </c>
-      <c r="X11" s="6" t="str">
+      <c r="W11" s="4" t="str">
+        <v/>
+      </c>
+      <c r="X11" s="4" t="str">
         <v>UNPLANNED</v>
       </c>
-      <c r="Y11" s="6" t="str">
-        <v/>
-      </c>
-      <c r="Z11" s="6" t="str">
+      <c r="Y11" s="4" t="str">
+        <v/>
+      </c>
+      <c r="Z11" s="4" t="str">
         <v>USA</v>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="8" t="str">
+      <c r="A12" s="4" t="str">
         <v>CDISCPILOT01</v>
       </c>
-      <c r="B12" s="8" t="str">
+      <c r="B12" s="4" t="str">
         <v>DM</v>
       </c>
-      <c r="C12" s="8" t="str">
+      <c r="C12" s="4" t="str">
         <v>CDISC008</v>
       </c>
-      <c r="D12" s="8">
+      <c r="D12" s="4">
         <v>1445</v>
       </c>
-      <c r="E12" s="10" t="str">
+      <c r="E12" s="6" t="str">
         <v>2014-05-11</v>
       </c>
-      <c r="F12" s="8" t="str">
+      <c r="F12" s="4" t="str">
         <v>2014-11-01</v>
       </c>
-      <c r="G12" s="8" t="str">
+      <c r="G12" s="4" t="str">
         <v>2014-05-11</v>
       </c>
-      <c r="H12" s="8" t="str">
+      <c r="H12" s="4" t="str">
         <v>2014-11-01</v>
       </c>
-      <c r="I12" s="8" t="str">
+      <c r="I12" s="4" t="str">
         <v>2014-05-01</v>
       </c>
-      <c r="J12" s="8" t="str">
+      <c r="J12" s="4" t="str">
         <v>2014-11-01</v>
       </c>
-      <c r="K12" s="8" t="str">
+      <c r="K12" s="4" t="str">
         <v>2014-11-01</v>
       </c>
-      <c r="L12" s="8" t="str">
+      <c r="L12" s="4" t="str">
         <v>Y</v>
       </c>
-      <c r="M12" s="8">
+      <c r="M12" s="4">
         <v>704</v>
       </c>
-      <c r="N12" s="8">
+      <c r="N12" s="4">
         <v>1939</v>
       </c>
-      <c r="O12" s="8">
+      <c r="O12" s="4">
         <v>75</v>
       </c>
-      <c r="P12" s="8" t="str">
+      <c r="P12" s="4" t="str">
         <v>YEARS</v>
       </c>
-      <c r="Q12" s="8" t="str">
+      <c r="Q12" s="4" t="str">
         <v>M</v>
       </c>
-      <c r="R12" s="8" t="str">
+      <c r="R12" s="4" t="str">
         <v>MULTIPLE</v>
       </c>
-      <c r="S12" s="8" t="str">
+      <c r="S12" s="4" t="str">
         <v>NOT HISPANIC OR LATINO</v>
       </c>
-      <c r="T12" s="8" t="str">
+      <c r="T12" s="4" t="str">
         <v>PLACEBO</v>
       </c>
-      <c r="U12" s="8" t="str">
+      <c r="U12" s="4" t="str">
         <v>Placebo</v>
       </c>
-      <c r="V12" s="8" t="str">
+      <c r="V12" s="4" t="str">
         <v>PLACEBO</v>
       </c>
-      <c r="W12" s="8" t="str">
+      <c r="W12" s="4" t="str">
         <v>Placebo</v>
       </c>
-      <c r="X12" s="8" t="str">
-        <v/>
-      </c>
-      <c r="Y12" s="8" t="str">
-        <v/>
-      </c>
-      <c r="Z12" s="8" t="str">
+      <c r="X12" s="4" t="str">
+        <v/>
+      </c>
+      <c r="Y12" s="4" t="str">
+        <v/>
+      </c>
+      <c r="Z12" s="4" t="str">
         <v>USA</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="6" t="str">
+      <c r="A13" s="4" t="str">
         <v>CDISCPILOT01</v>
       </c>
-      <c r="B13" s="6" t="str">
+      <c r="B13" s="4" t="str">
         <v>DM</v>
       </c>
-      <c r="C13" s="6" t="str">
+      <c r="C13" s="4" t="str">
         <v>CDISC009</v>
       </c>
-      <c r="D13" s="6">
+      <c r="D13" s="4">
         <v>1087</v>
       </c>
-      <c r="E13" s="6" t="str">
-        <v/>
-      </c>
-      <c r="F13" s="6" t="str">
+      <c r="E13" s="4" t="str">
+        <v/>
+      </c>
+      <c r="F13" s="4" t="str">
         <v>2013-04-28</v>
       </c>
-      <c r="G13" s="6" t="str">
+      <c r="G13" s="4" t="str">
         <v>2012-10-22</v>
       </c>
-      <c r="H13" s="6" t="str">
+      <c r="H13" s="4" t="str">
         <v>2013-04-28</v>
       </c>
-      <c r="I13" s="6" t="str">
+      <c r="I13" s="4" t="str">
         <v>2012-10-06</v>
       </c>
-      <c r="J13" s="6" t="str">
+      <c r="J13" s="4" t="str">
         <v>2013-04-28</v>
       </c>
-      <c r="K13" s="2" t="str">
-        <v/>
-      </c>
-      <c r="L13" s="6" t="str">
-        <v/>
-      </c>
-      <c r="M13" s="6">
+      <c r="K13" s="4" t="str">
+        <v/>
+      </c>
+      <c r="L13" s="4" t="str">
+        <v/>
+      </c>
+      <c r="M13" s="4">
         <v>708</v>
       </c>
-      <c r="N13" s="6">
+      <c r="N13" s="4">
         <v>1938</v>
       </c>
-      <c r="O13" s="6">
+      <c r="O13" s="4">
         <v>74</v>
       </c>
-      <c r="P13" s="6" t="str">
+      <c r="P13" s="4" t="str">
         <v>YEARS</v>
       </c>
-      <c r="Q13" s="6" t="str">
+      <c r="Q13" s="4" t="str">
         <v>F</v>
       </c>
-      <c r="R13" s="6" t="str">
+      <c r="R13" s="4" t="str">
         <v>WHITE</v>
       </c>
-      <c r="S13" s="6" t="str">
+      <c r="S13" s="4" t="str">
         <v>NOT HISPANIC OR LATINO</v>
       </c>
-      <c r="T13" s="6" t="str">
+      <c r="T13" s="4" t="str">
         <v>PLACEBO</v>
       </c>
-      <c r="U13" s="6" t="str">
+      <c r="U13" s="4" t="str">
         <v>Placebo</v>
       </c>
-      <c r="V13" s="6" t="str">
+      <c r="V13" s="4" t="str">
         <v>PLACEBO</v>
       </c>
-      <c r="W13" s="6" t="str">
+      <c r="W13" s="4" t="str">
         <v>Placebo</v>
       </c>
-      <c r="X13" s="6" t="str">
-        <v/>
-      </c>
-      <c r="Y13" s="6" t="str">
-        <v/>
-      </c>
-      <c r="Z13" s="6" t="str">
+      <c r="X13" s="4" t="str">
+        <v/>
+      </c>
+      <c r="Y13" s="4" t="str">
+        <v/>
+      </c>
+      <c r="Z13" s="4" t="str">
         <v>USA</v>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="8" t="str">
+      <c r="A14" s="4" t="str">
         <v>CDISCPILOT01</v>
       </c>
-      <c r="B14" s="8" t="str">
+      <c r="B14" s="4" t="str">
         <v>DM</v>
       </c>
-      <c r="C14" s="8" t="str">
+      <c r="C14" s="4" t="str">
         <v>CDISC010</v>
       </c>
-      <c r="D14" s="8">
+      <c r="D14" s="4">
         <v>1236</v>
       </c>
-      <c r="E14" s="10" t="str">
+      <c r="E14" s="6" t="str">
         <v>2013-09-21</v>
       </c>
-      <c r="F14" s="8" t="str">
+      <c r="F14" s="4" t="str">
         <v>2013-09-26</v>
       </c>
-      <c r="G14" s="8" t="str">
+      <c r="G14" s="4" t="str">
         <v>2013-09-21</v>
       </c>
-      <c r="H14" s="8" t="str">
+      <c r="H14" s="4" t="str">
         <v>2013-09-21</v>
       </c>
-      <c r="I14" s="8" t="str">
+      <c r="I14" s="4" t="str">
         <v>2013-09-08</v>
       </c>
-      <c r="J14" s="8" t="str">
+      <c r="J14" s="4" t="str">
         <v>2013-09-26</v>
       </c>
-      <c r="K14" s="8" t="str">
-        <v/>
-      </c>
-      <c r="L14" s="8" t="str">
-        <v/>
-      </c>
-      <c r="M14" s="8">
+      <c r="K14" s="4" t="str">
+        <v/>
+      </c>
+      <c r="L14" s="4" t="str">
+        <v/>
+      </c>
+      <c r="M14" s="4">
         <v>708</v>
       </c>
-      <c r="N14" s="8">
+      <c r="N14" s="4">
         <v>1927</v>
       </c>
-      <c r="O14" s="8">
+      <c r="O14" s="4">
         <v>86</v>
       </c>
-      <c r="P14" s="8" t="str">
+      <c r="P14" s="4" t="str">
         <v>YEARS</v>
       </c>
-      <c r="Q14" s="8" t="str">
+      <c r="Q14" s="4" t="str">
         <v>F</v>
       </c>
-      <c r="R14" s="8" t="str">
+      <c r="R14" s="4" t="str">
         <v>WHITE</v>
       </c>
-      <c r="S14" s="8" t="str">
+      <c r="S14" s="4" t="str">
         <v>NOT HISPANIC OR LATINO</v>
       </c>
-      <c r="T14" s="8" t="str">
+      <c r="T14" s="4" t="str">
         <v>ZAN_HIGH</v>
       </c>
-      <c r="U14" s="8" t="str">
+      <c r="U14" s="4" t="str">
         <v>Zanomaline High Dose (81 mg)</v>
       </c>
-      <c r="V14" s="8" t="str">
+      <c r="V14" s="4" t="str">
         <v>ZAN_HIGH</v>
       </c>
-      <c r="W14" s="8" t="str">
+      <c r="W14" s="4" t="str">
         <v>Zanomaline High Dose (81 mg)</v>
       </c>
-      <c r="X14" s="8" t="str">
-        <v/>
-      </c>
-      <c r="Y14" s="8" t="str">
-        <v/>
-      </c>
-      <c r="Z14" s="8" t="str">
+      <c r="X14" s="4" t="str">
+        <v/>
+      </c>
+      <c r="Y14" s="4" t="str">
+        <v/>
+      </c>
+      <c r="Z14" s="4" t="str">
         <v>USA</v>
       </c>
     </row>
@@ -2117,532 +2123,532 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="8" t="str">
+      <c r="A5" s="4" t="str">
         <v>CDISCPILOT01</v>
       </c>
-      <c r="B5" s="8" t="str">
+      <c r="B5" s="4" t="str">
         <v>CM</v>
       </c>
-      <c r="C5" s="8" t="str">
+      <c r="C5" s="4" t="str">
         <v>CDISC001</v>
       </c>
-      <c r="D5" s="8">
+      <c r="D5" s="4">
         <v>1</v>
       </c>
-      <c r="E5" s="8" t="str">
+      <c r="E5" s="4" t="str">
         <v>VITAMIN C</v>
       </c>
-      <c r="F5" s="8" t="str">
+      <c r="F5" s="4" t="str">
         <v>PROPHYLAXIS OR NON-THERAPEUTIC USE</v>
       </c>
-      <c r="G5" s="8">
+      <c r="G5" s="4">
         <v>500</v>
       </c>
-      <c r="H5" s="8" t="str">
+      <c r="H5" s="4" t="str">
         <v>mg</v>
       </c>
-      <c r="I5" s="8" t="str">
-        <v/>
-      </c>
-      <c r="J5" s="8" t="str">
+      <c r="I5" s="4" t="str">
+        <v/>
+      </c>
+      <c r="J5" s="4" t="str">
         <v>ORAL</v>
       </c>
-      <c r="K5" s="8" t="str">
+      <c r="K5" s="4" t="str">
         <v>SCREENING</v>
       </c>
-      <c r="L5" s="8">
+      <c r="L5" s="4">
         <v>1983</v>
       </c>
-      <c r="M5" s="8" t="str">
-        <v/>
-      </c>
-      <c r="N5" s="8" t="str">
-        <v/>
-      </c>
-      <c r="O5" s="8" t="str">
-        <v/>
-      </c>
-      <c r="P5" s="8" t="str">
-        <v/>
-      </c>
-      <c r="Q5" s="8" t="str">
+      <c r="M5" s="4" t="str">
+        <v/>
+      </c>
+      <c r="N5" s="4" t="str">
+        <v/>
+      </c>
+      <c r="O5" s="4" t="str">
+        <v/>
+      </c>
+      <c r="P5" s="4" t="str">
+        <v/>
+      </c>
+      <c r="Q5" s="4" t="str">
         <v>AFTER</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="6" t="str">
+      <c r="A6" s="4" t="str">
         <v>CDISCPILOT01</v>
       </c>
-      <c r="B6" s="6" t="str">
+      <c r="B6" s="4" t="str">
         <v>CM</v>
       </c>
-      <c r="C6" s="6" t="str">
+      <c r="C6" s="4" t="str">
         <v>CDISC002</v>
       </c>
-      <c r="D6" s="6">
+      <c r="D6" s="4">
         <v>2</v>
       </c>
-      <c r="E6" s="6" t="str">
+      <c r="E6" s="4" t="str">
         <v>VITAMIN E</v>
       </c>
-      <c r="F6" s="6" t="str">
+      <c r="F6" s="4" t="str">
         <v>PROPHYLAXIS OR NON-THERAPEUTIC USE</v>
       </c>
-      <c r="G6" s="6">
+      <c r="G6" s="4">
         <v>400</v>
       </c>
-      <c r="H6" s="6" t="str">
+      <c r="H6" s="4" t="str">
         <v>mg</v>
       </c>
-      <c r="I6" s="6" t="str">
-        <v/>
-      </c>
-      <c r="J6" s="6" t="str">
+      <c r="I6" s="4" t="str">
+        <v/>
+      </c>
+      <c r="J6" s="4" t="str">
         <v>ORAL</v>
       </c>
-      <c r="K6" s="6" t="str">
+      <c r="K6" s="4" t="str">
         <v>SCREENING</v>
       </c>
-      <c r="L6" s="6">
+      <c r="L6" s="4">
         <v>1983</v>
       </c>
-      <c r="M6" s="6" t="str">
-        <v/>
-      </c>
-      <c r="N6" s="6" t="str">
-        <v/>
-      </c>
-      <c r="O6" s="6" t="str">
-        <v/>
-      </c>
-      <c r="P6" s="6" t="str">
+      <c r="M6" s="4" t="str">
+        <v/>
+      </c>
+      <c r="N6" s="4" t="str">
+        <v/>
+      </c>
+      <c r="O6" s="4" t="str">
+        <v/>
+      </c>
+      <c r="P6" s="4" t="str">
         <v>ONGOING</v>
       </c>
-      <c r="Q6" s="6" t="str">
+      <c r="Q6" s="4" t="str">
         <v>AFTER</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="8" t="str">
+      <c r="A7" s="4" t="str">
         <v>CDISCPILOT01</v>
       </c>
-      <c r="B7" s="8" t="str">
+      <c r="B7" s="4" t="str">
         <v>CM</v>
       </c>
-      <c r="C7" s="8" t="str">
+      <c r="C7" s="4" t="str">
         <v>CDISC003</v>
       </c>
-      <c r="D7" s="8">
+      <c r="D7" s="4">
         <v>1</v>
       </c>
-      <c r="E7" s="8" t="str">
+      <c r="E7" s="4" t="str">
         <v>METAMUCIL</v>
       </c>
-      <c r="F7" s="8" t="str">
+      <c r="F7" s="4" t="str">
         <v>PROPHYLAXIS OR NON-THERAPEUTIC USE</v>
       </c>
-      <c r="G7" s="8">
+      <c r="G7" s="4">
         <v>3</v>
       </c>
-      <c r="H7" s="8" t="str">
+      <c r="H7" s="4" t="str">
         <v>mg</v>
       </c>
-      <c r="I7" s="8" t="str">
-        <v/>
-      </c>
-      <c r="J7" s="8" t="str">
+      <c r="I7" s="4" t="str">
+        <v/>
+      </c>
+      <c r="J7" s="4" t="str">
         <v>ORAL</v>
       </c>
-      <c r="K7" s="8" t="str">
+      <c r="K7" s="4" t="str">
         <v>SCREENING</v>
       </c>
-      <c r="L7" s="8">
+      <c r="L7" s="4">
         <v>2009</v>
       </c>
-      <c r="M7" s="8" t="str">
-        <v/>
-      </c>
-      <c r="N7" s="8" t="str">
-        <v/>
-      </c>
-      <c r="O7" s="8" t="str">
-        <v/>
-      </c>
-      <c r="P7" s="8" t="str">
-        <v/>
-      </c>
-      <c r="Q7" s="8" t="str">
+      <c r="M7" s="4" t="str">
+        <v/>
+      </c>
+      <c r="N7" s="4" t="str">
+        <v/>
+      </c>
+      <c r="O7" s="4" t="str">
+        <v/>
+      </c>
+      <c r="P7" s="4" t="str">
+        <v/>
+      </c>
+      <c r="Q7" s="4" t="str">
         <v/>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="6" t="str">
+      <c r="A8" s="4" t="str">
         <v>CDISCPILOT01</v>
       </c>
-      <c r="B8" s="6" t="str">
+      <c r="B8" s="4" t="str">
         <v>CM</v>
       </c>
-      <c r="C8" s="6" t="str">
+      <c r="C8" s="4" t="str">
         <v>CDISC004</v>
       </c>
-      <c r="D8" s="6">
+      <c r="D8" s="4">
         <v>2</v>
       </c>
-      <c r="E8" s="6" t="str">
+      <c r="E8" s="4" t="str">
         <v>ADVIL</v>
       </c>
-      <c r="F8" s="6" t="str">
+      <c r="F8" s="4" t="str">
         <v>PROPHYLAXIS OR NON-THERAPEUTIC USE</v>
       </c>
-      <c r="G8" s="6">
+      <c r="G8" s="4">
         <v>200</v>
       </c>
-      <c r="H8" s="6" t="str">
+      <c r="H8" s="4" t="str">
         <v>mg</v>
       </c>
-      <c r="I8" s="6" t="str">
-        <v/>
-      </c>
-      <c r="J8" s="6" t="str">
+      <c r="I8" s="4" t="str">
+        <v/>
+      </c>
+      <c r="J8" s="4" t="str">
         <v>ORAL</v>
       </c>
-      <c r="K8" s="6" t="str">
+      <c r="K8" s="4" t="str">
         <v>SCREENING</v>
       </c>
-      <c r="L8" s="6">
+      <c r="L8" s="4">
         <v>2011</v>
       </c>
-      <c r="M8" s="6" t="str">
-        <v/>
-      </c>
-      <c r="N8" s="6" t="str">
-        <v/>
-      </c>
-      <c r="O8" s="6" t="str">
-        <v/>
-      </c>
-      <c r="P8" s="6" t="str">
+      <c r="M8" s="4" t="str">
+        <v/>
+      </c>
+      <c r="N8" s="4" t="str">
+        <v/>
+      </c>
+      <c r="O8" s="4" t="str">
+        <v/>
+      </c>
+      <c r="P8" s="4" t="str">
         <v>ONGOING</v>
       </c>
-      <c r="Q8" s="6" t="str">
+      <c r="Q8" s="4" t="str">
         <v>AFTER</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="8" t="str">
+      <c r="A9" s="4" t="str">
         <v>CDISCPILOT01</v>
       </c>
-      <c r="B9" s="8" t="str">
+      <c r="B9" s="4" t="str">
         <v>CM</v>
       </c>
-      <c r="C9" s="8" t="str">
+      <c r="C9" s="4" t="str">
         <v>CDISC005</v>
       </c>
-      <c r="D9" s="8">
+      <c r="D9" s="4">
         <v>3</v>
       </c>
-      <c r="E9" s="8" t="str">
+      <c r="E9" s="4" t="str">
         <v>DOCUSATE SODIUM</v>
       </c>
-      <c r="F9" s="8" t="str">
+      <c r="F9" s="4" t="str">
         <v>PROPHYLAXIS OR NON-THERAPEUTIC USE</v>
       </c>
-      <c r="G9" s="8">
+      <c r="G9" s="4">
         <v>100</v>
       </c>
-      <c r="H9" s="8" t="str">
+      <c r="H9" s="4" t="str">
         <v>mg</v>
       </c>
-      <c r="I9" s="8" t="str">
-        <v/>
-      </c>
-      <c r="J9" s="8" t="str">
+      <c r="I9" s="4" t="str">
+        <v/>
+      </c>
+      <c r="J9" s="4" t="str">
         <v>ORAL</v>
       </c>
-      <c r="K9" s="8" t="str">
+      <c r="K9" s="4" t="str">
         <v>SCREENING</v>
       </c>
-      <c r="L9" s="8" t="str">
+      <c r="L9" s="4" t="str">
         <v>2012-11</v>
       </c>
-      <c r="M9" s="8" t="str">
+      <c r="M9" s="4" t="str">
         <v>2013-01-05</v>
       </c>
-      <c r="N9" s="8" t="str">
-        <v/>
-      </c>
-      <c r="O9" s="8">
+      <c r="N9" s="4" t="str">
+        <v/>
+      </c>
+      <c r="O9" s="4">
         <v>1</v>
       </c>
-      <c r="P9" s="8" t="str">
-        <v/>
-      </c>
-      <c r="Q9" s="8" t="str">
+      <c r="P9" s="4" t="str">
+        <v/>
+      </c>
+      <c r="Q9" s="4" t="str">
         <v/>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="6" t="str">
+      <c r="A10" s="4" t="str">
         <v>CDISCPILOT01</v>
       </c>
-      <c r="B10" s="6" t="str">
+      <c r="B10" s="4" t="str">
         <v>CM</v>
       </c>
-      <c r="C10" s="6" t="str">
+      <c r="C10" s="4" t="str">
         <v>CDISC006</v>
       </c>
-      <c r="D10" s="6">
+      <c r="D10" s="4">
         <v>4</v>
       </c>
-      <c r="E10" s="6" t="str">
+      <c r="E10" s="4" t="str">
         <v>BENADRYL</v>
       </c>
-      <c r="F10" s="6" t="str">
+      <c r="F10" s="4" t="str">
         <v>PROPHYLAXIS OR NON-THERAPEUTIC USE</v>
       </c>
-      <c r="G10" s="6">
+      <c r="G10" s="4">
         <v>75</v>
       </c>
-      <c r="H10" s="6" t="str">
+      <c r="H10" s="4" t="str">
         <v>mg</v>
       </c>
-      <c r="I10" s="6" t="str">
-        <v/>
-      </c>
-      <c r="J10" s="6" t="str">
+      <c r="I10" s="4" t="str">
+        <v/>
+      </c>
+      <c r="J10" s="4" t="str">
         <v>ORAL</v>
       </c>
-      <c r="K10" s="6" t="str">
+      <c r="K10" s="4" t="str">
         <v>SCREENING</v>
       </c>
-      <c r="L10" s="6" t="str">
+      <c r="L10" s="4" t="str">
         <v>2013-02-18</v>
       </c>
-      <c r="M10" s="6" t="str">
+      <c r="M10" s="4" t="str">
         <v>2013-05-10</v>
       </c>
-      <c r="N10" s="6">
+      <c r="N10" s="4">
         <v>45</v>
       </c>
-      <c r="O10" s="6">
+      <c r="O10" s="4">
         <v>126</v>
       </c>
-      <c r="P10" s="6" t="str">
-        <v/>
-      </c>
-      <c r="Q10" s="6" t="str">
+      <c r="P10" s="4" t="str">
+        <v/>
+      </c>
+      <c r="Q10" s="4" t="str">
         <v>AFTER</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="8" t="str">
+      <c r="A11" s="4" t="str">
         <v>CDISCPILOT01</v>
       </c>
-      <c r="B11" s="8" t="str">
+      <c r="B11" s="4" t="str">
         <v>CM</v>
       </c>
-      <c r="C11" s="8" t="str">
+      <c r="C11" s="4" t="str">
         <v>CDISC007</v>
       </c>
-      <c r="D11" s="8">
+      <c r="D11" s="4">
         <v>5</v>
       </c>
-      <c r="E11" s="8" t="str">
+      <c r="E11" s="4" t="str">
         <v>PREDNISONE</v>
       </c>
-      <c r="F11" s="8" t="str">
+      <c r="F11" s="4" t="str">
         <v>PROPHYLAXIS OR NON-THERAPEUTIC USE</v>
       </c>
-      <c r="G11" s="8">
+      <c r="G11" s="4">
         <v>20</v>
       </c>
-      <c r="H11" s="8" t="str">
+      <c r="H11" s="4" t="str">
         <v>mg</v>
       </c>
-      <c r="I11" s="8" t="str">
-        <v/>
-      </c>
-      <c r="J11" s="8" t="str">
+      <c r="I11" s="4" t="str">
+        <v/>
+      </c>
+      <c r="J11" s="4" t="str">
         <v>ORAL</v>
       </c>
-      <c r="K11" s="8" t="str">
+      <c r="K11" s="4" t="str">
         <v>SCREENING</v>
       </c>
-      <c r="L11" s="10" t="str">
+      <c r="L11" s="6" t="str">
         <v>2013-02-18</v>
       </c>
-      <c r="M11" s="8" t="str">
+      <c r="M11" s="4" t="str">
         <v>2013-05-10</v>
       </c>
-      <c r="N11" s="9" t="str">
-        <v/>
-      </c>
-      <c r="O11" s="6">
+      <c r="N11" s="6" t="str">
+        <v/>
+      </c>
+      <c r="O11" s="4">
         <v>126</v>
       </c>
-      <c r="P11" s="8" t="str">
+      <c r="P11" s="4" t="str">
         <v>BEFORE</v>
       </c>
-      <c r="Q11" s="8" t="str">
+      <c r="Q11" s="4" t="str">
         <v/>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="6" t="str">
+      <c r="A12" s="4" t="str">
         <v>CDISCPILOT01</v>
       </c>
-      <c r="B12" s="6" t="str">
+      <c r="B12" s="4" t="str">
         <v>CM</v>
       </c>
-      <c r="C12" s="6" t="str">
+      <c r="C12" s="4" t="str">
         <v>CDISC008</v>
       </c>
-      <c r="D12" s="6">
+      <c r="D12" s="4">
         <v>6</v>
       </c>
-      <c r="E12" s="6" t="str">
+      <c r="E12" s="4" t="str">
         <v>TEMOVATE</v>
       </c>
-      <c r="F12" s="6" t="str">
+      <c r="F12" s="4" t="str">
         <v>PROPHYLAXIS OR NON-THERAPEUTIC USE</v>
       </c>
-      <c r="G12" s="6">
+      <c r="G12" s="4">
         <v>1</v>
       </c>
-      <c r="H12" s="6" t="str">
+      <c r="H12" s="4" t="str">
         <v>TABLET</v>
       </c>
-      <c r="I12" s="6" t="str">
-        <v/>
-      </c>
-      <c r="J12" s="6" t="str">
+      <c r="I12" s="4" t="str">
+        <v/>
+      </c>
+      <c r="J12" s="4" t="str">
         <v>TOPICAL</v>
       </c>
-      <c r="K12" s="6" t="str">
+      <c r="K12" s="4" t="str">
         <v>SCREENING</v>
       </c>
-      <c r="L12" s="10" t="str">
+      <c r="L12" s="6" t="str">
         <v>2013-02-18</v>
       </c>
-      <c r="M12" s="6" t="str">
+      <c r="M12" s="4" t="str">
         <v>2013-02-20</v>
       </c>
-      <c r="N12" s="11">
+      <c r="N12" s="6">
         <v>45</v>
       </c>
-      <c r="O12" s="6">
+      <c r="O12" s="4">
         <v>47</v>
       </c>
-      <c r="P12" s="6" t="str">
+      <c r="P12" s="4" t="str">
         <v>BEFORE</v>
       </c>
-      <c r="Q12" s="6" t="str">
+      <c r="Q12" s="4" t="str">
         <v/>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="8" t="str">
+      <c r="A13" s="4" t="str">
         <v>CDISCPILOT01</v>
       </c>
-      <c r="B13" s="8" t="str">
+      <c r="B13" s="4" t="str">
         <v>CM</v>
       </c>
-      <c r="C13" s="8" t="str">
+      <c r="C13" s="4" t="str">
         <v>CDISC009</v>
       </c>
-      <c r="D13" s="8">
+      <c r="D13" s="4">
         <v>1</v>
       </c>
-      <c r="E13" s="8" t="str">
+      <c r="E13" s="4" t="str">
         <v>MOTRIN</v>
       </c>
-      <c r="F13" s="8" t="str">
+      <c r="F13" s="4" t="str">
         <v>PROPHYLAXIS OR NON-THERAPEUTIC USE</v>
       </c>
-      <c r="G13" s="8">
+      <c r="G13" s="4">
         <v>400</v>
       </c>
-      <c r="H13" s="8" t="str">
+      <c r="H13" s="4" t="str">
         <v>mg</v>
       </c>
-      <c r="I13" s="8" t="str">
-        <v/>
-      </c>
-      <c r="J13" s="8" t="str">
+      <c r="I13" s="4" t="str">
+        <v/>
+      </c>
+      <c r="J13" s="4" t="str">
         <v>ORAL</v>
       </c>
-      <c r="K13" s="8" t="str">
+      <c r="K13" s="4" t="str">
         <v>SCREENING</v>
       </c>
-      <c r="L13" s="8" t="str">
+      <c r="L13" s="4" t="str">
         <v>1998-10</v>
       </c>
-      <c r="M13" s="8" t="str">
+      <c r="M13" s="4" t="str">
         <v>2013-06-05</v>
       </c>
-      <c r="N13" s="8" t="str">
-        <v/>
-      </c>
-      <c r="O13" s="8">
+      <c r="N13" s="4" t="str">
+        <v/>
+      </c>
+      <c r="O13" s="4">
         <v>181</v>
       </c>
-      <c r="P13" s="8" t="str">
-        <v/>
-      </c>
-      <c r="Q13" s="8" t="str">
+      <c r="P13" s="4" t="str">
+        <v/>
+      </c>
+      <c r="Q13" s="4" t="str">
         <v/>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="6" t="str">
+      <c r="A14" s="4" t="str">
         <v>CDISCPILOT01</v>
       </c>
-      <c r="B14" s="6" t="str">
+      <c r="B14" s="4" t="str">
         <v>CM</v>
       </c>
-      <c r="C14" s="6" t="str">
+      <c r="C14" s="4" t="str">
         <v>CDISC010</v>
       </c>
-      <c r="D14" s="6">
+      <c r="D14" s="4">
         <v>2</v>
       </c>
-      <c r="E14" s="6" t="str">
+      <c r="E14" s="4" t="str">
         <v>PRINIVIL</v>
       </c>
-      <c r="F14" s="6" t="str">
+      <c r="F14" s="4" t="str">
         <v>PROPHYLAXIS OR NON-THERAPEUTIC USE</v>
       </c>
-      <c r="G14" s="6">
+      <c r="G14" s="4">
         <v>10</v>
       </c>
-      <c r="H14" s="6" t="str">
+      <c r="H14" s="4" t="str">
         <v>mg</v>
       </c>
-      <c r="I14" s="6" t="str">
-        <v/>
-      </c>
-      <c r="J14" s="6" t="str">
+      <c r="I14" s="4" t="str">
+        <v/>
+      </c>
+      <c r="J14" s="4" t="str">
         <v>ORAL</v>
       </c>
-      <c r="K14" s="6" t="str">
+      <c r="K14" s="4" t="str">
         <v>SCREENING</v>
       </c>
-      <c r="L14" s="10" t="str">
+      <c r="L14" s="6" t="str">
         <v>2011-07-15</v>
       </c>
-      <c r="M14" s="6" t="str">
+      <c r="M14" s="4" t="str">
         <v>2013-06-05</v>
       </c>
-      <c r="N14" s="11">
+      <c r="N14" s="6">
         <v>-511</v>
       </c>
-      <c r="O14" s="6">
+      <c r="O14" s="4">
         <v>181</v>
       </c>
-      <c r="P14" s="6" t="str">
-        <v/>
-      </c>
-      <c r="Q14" s="6" t="str">
+      <c r="P14" s="4" t="str">
+        <v/>
+      </c>
+      <c r="Q14" s="4" t="str">
         <v/>
       </c>
     </row>

</xml_diff>